<commit_message>
Formato control de despachos reparado
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO CONTROL DE DESPACHO.xlsx
+++ b/storage/app/templates/FORMATO CONTROL DE DESPACHO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2785B3FE-A39C-437E-8765-3EF3DD9A31BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C23CD6D1-AE5A-4038-92EE-56BFBD8542C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="23">
   <si>
     <t>Fecha</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>{{fecha_retorno}}</t>
+  </si>
+  <si>
+    <t>Retorna (Si/No)</t>
   </si>
 </sst>
 </file>
@@ -307,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -424,14 +427,19 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -807,9 +815,9 @@
     <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="6.88671875" customWidth="1"/>
     <col min="9" max="9" width="25.6640625" customWidth="1"/>
-    <col min="10" max="10" width="9.109375" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" customWidth="1"/>
-    <col min="12" max="12" width="24.5546875" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" customWidth="1"/>
+    <col min="11" max="11" width="15.109375" customWidth="1"/>
+    <col min="12" max="12" width="19.5546875" customWidth="1"/>
     <col min="13" max="13" width="6.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -908,7 +916,7 @@
         <v>8</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>10</v>
@@ -918,598 +926,598 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32" t="s">
+      <c r="D7" s="31"/>
+      <c r="E7" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="30" t="s">
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="30" t="s">
+      <c r="I7" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="30" t="s">
+      <c r="J7" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="30" t="s">
+      <c r="K7" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="3"/>
+      <c r="L7" s="33"/>
     </row>
     <row r="8" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32" t="s">
+      <c r="D8" s="31"/>
+      <c r="E8" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="30" t="s">
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="I8" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J8" s="30" t="s">
+      <c r="J8" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="30" t="s">
+      <c r="K8" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="3"/>
+      <c r="L8" s="33"/>
     </row>
     <row r="9" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="30" t="s">
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="30" t="s">
+      <c r="I9" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="30" t="s">
+      <c r="J9" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="30" t="s">
+      <c r="K9" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L9" s="3"/>
+      <c r="L9" s="33"/>
     </row>
     <row r="10" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32" t="s">
+      <c r="D10" s="31"/>
+      <c r="E10" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="30" t="s">
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="30" t="s">
+      <c r="I10" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="30" t="s">
+      <c r="J10" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K10" s="30" t="s">
+      <c r="K10" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="3"/>
+      <c r="L10" s="33"/>
     </row>
     <row r="11" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32" t="s">
+      <c r="D11" s="31"/>
+      <c r="E11" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="30" t="s">
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="30" t="s">
+      <c r="I11" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="30" t="s">
+      <c r="J11" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="30" t="s">
+      <c r="K11" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L11" s="3"/>
+      <c r="L11" s="33"/>
     </row>
     <row r="12" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="31" t="s">
+      <c r="B12" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="C12" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32" t="s">
+      <c r="D12" s="31"/>
+      <c r="E12" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="30" t="s">
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="30" t="s">
+      <c r="I12" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="30" t="s">
+      <c r="J12" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K12" s="30" t="s">
+      <c r="K12" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L12" s="3"/>
+      <c r="L12" s="33"/>
     </row>
     <row r="13" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32" t="s">
+      <c r="D13" s="31"/>
+      <c r="E13" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="30" t="s">
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="30" t="s">
+      <c r="I13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="30" t="s">
+      <c r="J13" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K13" s="30" t="s">
+      <c r="K13" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="3"/>
+      <c r="L13" s="33"/>
     </row>
     <row r="14" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32" t="s">
+      <c r="D14" s="31"/>
+      <c r="E14" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="30" t="s">
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="30" t="s">
+      <c r="I14" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="30" t="s">
+      <c r="J14" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K14" s="30" t="s">
+      <c r="K14" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L14" s="3"/>
+      <c r="L14" s="33"/>
     </row>
     <row r="15" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32" t="s">
+      <c r="D15" s="31"/>
+      <c r="E15" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="30" t="s">
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="30" t="s">
+      <c r="I15" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="30" t="s">
+      <c r="J15" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K15" s="30" t="s">
+      <c r="K15" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L15" s="3"/>
+      <c r="L15" s="33"/>
     </row>
     <row r="16" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="C16" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32" t="s">
+      <c r="D16" s="31"/>
+      <c r="E16" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="30" t="s">
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="30" t="s">
+      <c r="I16" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="30" t="s">
+      <c r="J16" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K16" s="30" t="s">
+      <c r="K16" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L16" s="3"/>
+      <c r="L16" s="33"/>
     </row>
     <row r="17" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32" t="s">
+      <c r="D17" s="31"/>
+      <c r="E17" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="30" t="s">
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I17" s="30" t="s">
+      <c r="I17" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="30" t="s">
+      <c r="J17" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K17" s="30" t="s">
+      <c r="K17" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L17" s="3"/>
+      <c r="L17" s="33"/>
     </row>
     <row r="18" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32" t="s">
+      <c r="D18" s="31"/>
+      <c r="E18" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="30" t="s">
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="30" t="s">
+      <c r="I18" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="30" t="s">
+      <c r="J18" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K18" s="30" t="s">
+      <c r="K18" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L18" s="3"/>
+      <c r="L18" s="33"/>
     </row>
     <row r="19" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="32" t="s">
+      <c r="C19" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32" t="s">
+      <c r="D19" s="31"/>
+      <c r="E19" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="30" t="s">
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="30" t="s">
+      <c r="I19" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J19" s="30" t="s">
+      <c r="J19" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K19" s="30" t="s">
+      <c r="K19" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L19" s="3"/>
+      <c r="L19" s="33"/>
     </row>
     <row r="20" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="32" t="s">
+      <c r="C20" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32" t="s">
+      <c r="D20" s="31"/>
+      <c r="E20" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="30" t="s">
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="30" t="s">
+      <c r="I20" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="30" t="s">
+      <c r="J20" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K20" s="30" t="s">
+      <c r="K20" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L20" s="3"/>
+      <c r="L20" s="33"/>
     </row>
     <row r="21" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="32" t="s">
+      <c r="C21" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32" t="s">
+      <c r="D21" s="31"/>
+      <c r="E21" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="30" t="s">
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="30" t="s">
+      <c r="I21" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="30" t="s">
+      <c r="J21" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K21" s="30" t="s">
+      <c r="K21" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L21" s="3"/>
+      <c r="L21" s="33"/>
     </row>
     <row r="22" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32" t="s">
+      <c r="D22" s="31"/>
+      <c r="E22" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="30" t="s">
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="30" t="s">
+      <c r="I22" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J22" s="30" t="s">
+      <c r="J22" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K22" s="30" t="s">
+      <c r="K22" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L22" s="3"/>
+      <c r="L22" s="33"/>
     </row>
     <row r="23" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C23" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32" t="s">
+      <c r="D23" s="31"/>
+      <c r="E23" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="30" t="s">
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="30" t="s">
+      <c r="I23" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J23" s="30" t="s">
+      <c r="J23" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K23" s="30" t="s">
+      <c r="K23" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L23" s="3"/>
+      <c r="L23" s="33"/>
     </row>
     <row r="24" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32" t="s">
+      <c r="D24" s="31"/>
+      <c r="E24" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="30" t="s">
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I24" s="30" t="s">
+      <c r="I24" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J24" s="30" t="s">
+      <c r="J24" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K24" s="30" t="s">
+      <c r="K24" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L24" s="3"/>
+      <c r="L24" s="33"/>
     </row>
     <row r="25" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="32" t="s">
+      <c r="C25" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32" t="s">
+      <c r="D25" s="31"/>
+      <c r="E25" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="30" t="s">
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I25" s="30" t="s">
+      <c r="I25" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="30" t="s">
+      <c r="J25" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K25" s="30" t="s">
+      <c r="K25" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L25" s="3"/>
+      <c r="L25" s="33"/>
     </row>
     <row r="26" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="32" t="s">
+      <c r="C26" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32" t="s">
+      <c r="D26" s="31"/>
+      <c r="E26" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="30" t="s">
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I26" s="30" t="s">
+      <c r="I26" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J26" s="30" t="s">
+      <c r="J26" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K26" s="30" t="s">
+      <c r="K26" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L26" s="3"/>
+      <c r="L26" s="33"/>
     </row>
     <row r="27" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32" t="s">
+      <c r="D27" s="31"/>
+      <c r="E27" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="30" t="s">
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I27" s="30" t="s">
+      <c r="I27" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J27" s="30" t="s">
+      <c r="J27" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K27" s="30" t="s">
+      <c r="K27" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L27" s="3"/>
+      <c r="L27" s="33"/>
     </row>
     <row r="28" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="32" t="s">
+      <c r="C28" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32" t="s">
+      <c r="D28" s="31"/>
+      <c r="E28" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="30" t="s">
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="30" t="s">
+      <c r="I28" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="30" t="s">
+      <c r="J28" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="30" t="s">
+      <c r="K28" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="L28" s="3"/>
+      <c r="L28" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="53">

</xml_diff>

<commit_message>
Exportaciones de Sumarios y ODC hechas, mas modulo de informacion AGARCORP
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO CONTROL DE DESPACHO.xlsx
+++ b/storage/app/templates/FORMATO CONTROL DE DESPACHO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DECB52CE-936A-4042-B36A-B5B895C7701F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197294D8-DBF9-4F0E-8344-67D9670EC97C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -310,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -334,14 +334,26 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" indent="1"/>
       <protection locked="0"/>
@@ -386,18 +398,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -441,6 +441,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -464,31 +467,31 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>381001</xdr:colOff>
+      <xdr:colOff>348343</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>99361</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>466725</xdr:colOff>
+      <xdr:colOff>555172</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>185056</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 1">
+        <xdr:cNvPr id="6" name="Imagen 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C89C093F-C7CB-4A47-B3E4-9F608769EBEB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -502,16 +505,13 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="876301" y="171450"/>
-          <a:ext cx="904874" cy="657225"/>
+          <a:off x="555172" y="99361"/>
+          <a:ext cx="1088571" cy="902124"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
             <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
@@ -519,16 +519,6 @@
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
             </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
           </a:ext>
         </a:extLst>
       </xdr:spPr>
@@ -822,93 +812,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="11" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="9" t="s">
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="9"/>
+      <c r="L1" s="12"/>
     </row>
     <row r="2" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="9" t="s">
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="9"/>
+      <c r="L2" s="12"/>
     </row>
     <row r="3" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="9" t="s">
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="9"/>
+      <c r="L3" s="12"/>
     </row>
     <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="9" t="s">
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="9"/>
+      <c r="L4" s="12"/>
     </row>
     <row r="5" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
     </row>
     <row r="6" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="20" t="s">
+      <c r="D6" s="9"/>
+      <c r="E6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="9"/>
       <c r="H6" s="2" t="s">
         <v>7</v>
       </c>
@@ -929,15 +919,15 @@
       <c r="B7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8" t="s">
+      <c r="D7" s="10"/>
+      <c r="E7" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
       <c r="H7" s="5" t="s">
         <v>18</v>
       </c>
@@ -956,15 +946,15 @@
       <c r="B8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8" t="s">
+      <c r="D8" s="10"/>
+      <c r="E8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
       <c r="H8" s="5" t="s">
         <v>18</v>
       </c>
@@ -983,15 +973,15 @@
       <c r="B9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8" t="s">
+      <c r="D9" s="10"/>
+      <c r="E9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
       <c r="H9" s="5" t="s">
         <v>18</v>
       </c>
@@ -1010,15 +1000,15 @@
       <c r="B10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8" t="s">
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
       <c r="H10" s="5" t="s">
         <v>18</v>
       </c>
@@ -1037,15 +1027,15 @@
       <c r="B11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8" t="s">
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
       <c r="H11" s="5" t="s">
         <v>18</v>
       </c>
@@ -1064,15 +1054,15 @@
       <c r="B12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8" t="s">
+      <c r="D12" s="10"/>
+      <c r="E12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
       <c r="H12" s="5" t="s">
         <v>18</v>
       </c>
@@ -1091,15 +1081,15 @@
       <c r="B13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8" t="s">
+      <c r="D13" s="10"/>
+      <c r="E13" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
       <c r="H13" s="5" t="s">
         <v>18</v>
       </c>
@@ -1118,15 +1108,15 @@
       <c r="B14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8" t="s">
+      <c r="D14" s="10"/>
+      <c r="E14" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
       <c r="H14" s="5" t="s">
         <v>18</v>
       </c>
@@ -1145,15 +1135,15 @@
       <c r="B15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8" t="s">
+      <c r="D15" s="10"/>
+      <c r="E15" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
       <c r="H15" s="5" t="s">
         <v>18</v>
       </c>
@@ -1172,15 +1162,15 @@
       <c r="B16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8" t="s">
+      <c r="D16" s="10"/>
+      <c r="E16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
       <c r="H16" s="5" t="s">
         <v>18</v>
       </c>
@@ -1199,15 +1189,15 @@
       <c r="B17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8" t="s">
+      <c r="D17" s="10"/>
+      <c r="E17" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
       <c r="H17" s="5" t="s">
         <v>18</v>
       </c>
@@ -1226,15 +1216,15 @@
       <c r="B18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8" t="s">
+      <c r="D18" s="10"/>
+      <c r="E18" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
       <c r="H18" s="5" t="s">
         <v>18</v>
       </c>
@@ -1253,15 +1243,15 @@
       <c r="B19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8" t="s">
+      <c r="D19" s="10"/>
+      <c r="E19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
       <c r="H19" s="5" t="s">
         <v>18</v>
       </c>
@@ -1280,15 +1270,15 @@
       <c r="B20" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8" t="s">
+      <c r="D20" s="10"/>
+      <c r="E20" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
       <c r="H20" s="5" t="s">
         <v>18</v>
       </c>
@@ -1307,15 +1297,15 @@
       <c r="B21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8" t="s">
+      <c r="D21" s="10"/>
+      <c r="E21" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
       <c r="H21" s="5" t="s">
         <v>18</v>
       </c>
@@ -1334,15 +1324,15 @@
       <c r="B22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8" t="s">
+      <c r="D22" s="10"/>
+      <c r="E22" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
       <c r="H22" s="5" t="s">
         <v>18</v>
       </c>
@@ -1361,15 +1351,15 @@
       <c r="B23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8" t="s">
+      <c r="D23" s="10"/>
+      <c r="E23" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
       <c r="H23" s="5" t="s">
         <v>18</v>
       </c>
@@ -1388,15 +1378,15 @@
       <c r="B24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8" t="s">
+      <c r="D24" s="10"/>
+      <c r="E24" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
       <c r="H24" s="5" t="s">
         <v>18</v>
       </c>
@@ -1415,15 +1405,15 @@
       <c r="B25" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8" t="s">
+      <c r="D25" s="10"/>
+      <c r="E25" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
       <c r="H25" s="5" t="s">
         <v>18</v>
       </c>
@@ -1442,15 +1432,15 @@
       <c r="B26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8" t="s">
+      <c r="D26" s="10"/>
+      <c r="E26" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
       <c r="H26" s="5" t="s">
         <v>18</v>
       </c>
@@ -1469,15 +1459,15 @@
       <c r="B27" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8" t="s">
+      <c r="D27" s="10"/>
+      <c r="E27" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
       <c r="H27" s="5" t="s">
         <v>18</v>
       </c>
@@ -1496,15 +1486,15 @@
       <c r="B28" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8" t="s">
+      <c r="D28" s="10"/>
+      <c r="E28" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
       <c r="H28" s="5" t="s">
         <v>18</v>
       </c>
@@ -1521,20 +1511,29 @@
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B1:C4"/>
+    <mergeCell ref="D1:J4"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="C23:D23"/>
@@ -1551,29 +1550,20 @@
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="B5:L5"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="B1:C4"/>
-    <mergeCell ref="D1:J4"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E9:G9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19" right="0.16" top="0.63" bottom="0.56999999999999995" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -1616,10 +1606,10 @@
       <c r="H1" s="26"/>
       <c r="I1" s="26"/>
       <c r="J1" s="27"/>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="9"/>
+      <c r="L1" s="12"/>
     </row>
     <row r="2" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="28"/>
@@ -1631,10 +1621,10 @@
       <c r="H2" s="29"/>
       <c r="I2" s="29"/>
       <c r="J2" s="30"/>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="9"/>
+      <c r="L2" s="12"/>
     </row>
     <row r="3" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="28"/>
@@ -1646,10 +1636,10 @@
       <c r="H3" s="29"/>
       <c r="I3" s="29"/>
       <c r="J3" s="30"/>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="9"/>
+      <c r="L3" s="12"/>
     </row>
     <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="31"/>
@@ -1661,37 +1651,37 @@
       <c r="H4" s="32"/>
       <c r="I4" s="32"/>
       <c r="J4" s="33"/>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="9"/>
+      <c r="L4" s="12"/>
     </row>
     <row r="5" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
     </row>
     <row r="6" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="20" t="s">
+      <c r="D6" s="9"/>
+      <c r="E6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="9"/>
       <c r="H6" s="2" t="s">
         <v>7</v>
       </c>
@@ -1713,7 +1703,7 @@
       <c r="C7" s="23"/>
       <c r="D7" s="24"/>
       <c r="E7" s="23"/>
-      <c r="F7" s="7"/>
+      <c r="F7" s="11"/>
       <c r="G7" s="24"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -1726,7 +1716,7 @@
       <c r="C8" s="23"/>
       <c r="D8" s="24"/>
       <c r="E8" s="23"/>
-      <c r="F8" s="7"/>
+      <c r="F8" s="11"/>
       <c r="G8" s="24"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -1741,7 +1731,7 @@
       </c>
       <c r="D9" s="24"/>
       <c r="E9" s="23"/>
-      <c r="F9" s="7"/>
+      <c r="F9" s="11"/>
       <c r="G9" s="24"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -1754,7 +1744,7 @@
       <c r="C10" s="23"/>
       <c r="D10" s="24"/>
       <c r="E10" s="23"/>
-      <c r="F10" s="7"/>
+      <c r="F10" s="11"/>
       <c r="G10" s="24"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -1767,7 +1757,7 @@
       <c r="C11" s="23"/>
       <c r="D11" s="24"/>
       <c r="E11" s="23"/>
-      <c r="F11" s="7"/>
+      <c r="F11" s="11"/>
       <c r="G11" s="24"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -1780,7 +1770,7 @@
       <c r="C12" s="23"/>
       <c r="D12" s="24"/>
       <c r="E12" s="23"/>
-      <c r="F12" s="7"/>
+      <c r="F12" s="11"/>
       <c r="G12" s="24"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -1793,7 +1783,7 @@
       <c r="C13" s="23"/>
       <c r="D13" s="24"/>
       <c r="E13" s="23"/>
-      <c r="F13" s="7"/>
+      <c r="F13" s="11"/>
       <c r="G13" s="24"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -1806,7 +1796,7 @@
       <c r="C14" s="23"/>
       <c r="D14" s="24"/>
       <c r="E14" s="23"/>
-      <c r="F14" s="7"/>
+      <c r="F14" s="11"/>
       <c r="G14" s="24"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -1819,7 +1809,7 @@
       <c r="C15" s="23"/>
       <c r="D15" s="24"/>
       <c r="E15" s="23"/>
-      <c r="F15" s="7"/>
+      <c r="F15" s="11"/>
       <c r="G15" s="24"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -1834,7 +1824,7 @@
       <c r="C16" s="23"/>
       <c r="D16" s="24"/>
       <c r="E16" s="23"/>
-      <c r="F16" s="7"/>
+      <c r="F16" s="11"/>
       <c r="G16" s="24"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -1847,7 +1837,7 @@
       <c r="C17" s="23"/>
       <c r="D17" s="24"/>
       <c r="E17" s="23"/>
-      <c r="F17" s="7"/>
+      <c r="F17" s="11"/>
       <c r="G17" s="24"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -1860,7 +1850,7 @@
       <c r="C18" s="23"/>
       <c r="D18" s="24"/>
       <c r="E18" s="23"/>
-      <c r="F18" s="7"/>
+      <c r="F18" s="11"/>
       <c r="G18" s="24"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -1873,7 +1863,7 @@
       <c r="C19" s="23"/>
       <c r="D19" s="24"/>
       <c r="E19" s="23"/>
-      <c r="F19" s="7"/>
+      <c r="F19" s="11"/>
       <c r="G19" s="24"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -1886,7 +1876,7 @@
       <c r="C20" s="23"/>
       <c r="D20" s="24"/>
       <c r="E20" s="23"/>
-      <c r="F20" s="7"/>
+      <c r="F20" s="11"/>
       <c r="G20" s="24"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
@@ -1899,7 +1889,7 @@
       <c r="C21" s="23"/>
       <c r="D21" s="24"/>
       <c r="E21" s="23"/>
-      <c r="F21" s="7"/>
+      <c r="F21" s="11"/>
       <c r="G21" s="24"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
@@ -1912,7 +1902,7 @@
       <c r="C22" s="23"/>
       <c r="D22" s="24"/>
       <c r="E22" s="23"/>
-      <c r="F22" s="7"/>
+      <c r="F22" s="11"/>
       <c r="G22" s="24"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
@@ -1925,7 +1915,7 @@
       <c r="C23" s="23"/>
       <c r="D23" s="24"/>
       <c r="E23" s="23"/>
-      <c r="F23" s="7"/>
+      <c r="F23" s="11"/>
       <c r="G23" s="24"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
@@ -1938,7 +1928,7 @@
       <c r="C24" s="23"/>
       <c r="D24" s="24"/>
       <c r="E24" s="23"/>
-      <c r="F24" s="7"/>
+      <c r="F24" s="11"/>
       <c r="G24" s="24"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
@@ -1951,7 +1941,7 @@
       <c r="C25" s="23"/>
       <c r="D25" s="24"/>
       <c r="E25" s="23"/>
-      <c r="F25" s="7"/>
+      <c r="F25" s="11"/>
       <c r="G25" s="24"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
@@ -1964,7 +1954,7 @@
       <c r="C26" s="23"/>
       <c r="D26" s="24"/>
       <c r="E26" s="23"/>
-      <c r="F26" s="7"/>
+      <c r="F26" s="11"/>
       <c r="G26" s="24"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
@@ -1977,7 +1967,7 @@
       <c r="C27" s="23"/>
       <c r="D27" s="24"/>
       <c r="E27" s="23"/>
-      <c r="F27" s="7"/>
+      <c r="F27" s="11"/>
       <c r="G27" s="24"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
@@ -1987,10 +1977,10 @@
     </row>
     <row r="28" spans="2:12" ht="24.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
       <c r="E28" s="23"/>
-      <c r="F28" s="7"/>
+      <c r="F28" s="11"/>
       <c r="G28" s="24"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -2000,11 +1990,475 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:G20"/>
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="C28:D28"/>
     <mergeCell ref="E28:G28"/>
     <mergeCell ref="B1:J4"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="C23:D23"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.19" right="0.16" top="0.63" bottom="0.56999999999999995" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup scale="81" orientation="landscape" copies="2" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2B83C57-79D2-4FE4-AEF0-9E768795144B}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:L28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="7" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" customWidth="1"/>
+    <col min="10" max="10" width="7.6640625" customWidth="1"/>
+    <col min="11" max="11" width="10.109375" customWidth="1"/>
+    <col min="12" max="12" width="15.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="16"/>
+    </row>
+    <row r="2" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="17"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="19"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="19"/>
+    </row>
+    <row r="4" spans="2:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="20"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="22"/>
+    </row>
+    <row r="5" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+    </row>
+    <row r="6" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="3"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+    </row>
+    <row r="8" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="3"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="3"/>
+      <c r="C9" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="24"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="3"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="3"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="3"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="3"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="3"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="3"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="3"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="3"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="3"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="3"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+    </row>
+    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="3"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+    </row>
+    <row r="21" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="3"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="3"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+    </row>
+    <row r="23" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="3"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+    </row>
+    <row r="24" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="3"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+    </row>
+    <row r="25" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="3"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="3"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+    </row>
+    <row r="27" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="3"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+    </row>
+    <row r="28" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="3"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="48">
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="B1:L4"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="C25:D25"/>
@@ -2043,10 +2497,6 @@
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:G8"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E6:G6"/>
@@ -2054,466 +2504,6 @@
     <mergeCell ref="E7:G7"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.19" right="0.16" top="0.63" bottom="0.56999999999999995" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="81" orientation="landscape" copies="2" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2B83C57-79D2-4FE4-AEF0-9E768795144B}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B1:L28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="10.6640625" customWidth="1"/>
-    <col min="3" max="7" width="12.6640625" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" customWidth="1"/>
-    <col min="11" max="11" width="10.109375" customWidth="1"/>
-    <col min="12" max="12" width="15.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="13"/>
-    </row>
-    <row r="2" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="14"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="16"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="14"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="16"/>
-    </row>
-    <row r="4" spans="2:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="19"/>
-    </row>
-    <row r="5" spans="2:12" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-    </row>
-    <row r="6" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="3"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="3"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="3"/>
-      <c r="C9" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="24"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="3"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="3"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="3"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="3"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-    </row>
-    <row r="14" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="3"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-    </row>
-    <row r="15" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="3"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L15" s="3"/>
-    </row>
-    <row r="16" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="3"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="2:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="3"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="3"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-    </row>
-    <row r="19" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="3"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-    </row>
-    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="3"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-    </row>
-    <row r="21" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="3"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-    </row>
-    <row r="22" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="3"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="3"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-    </row>
-    <row r="24" spans="2:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="3"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
-    </row>
-    <row r="25" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="3"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
-    </row>
-    <row r="26" spans="2:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="3"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-    </row>
-    <row r="27" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="3"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-    </row>
-    <row r="28" spans="2:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="3"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-    </row>
-  </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="B5:L5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="B1:L4"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="C23:D23"/>
-  </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="93" orientation="landscape" copies="2" r:id="rId1"/>
 </worksheet>

</xml_diff>